<commit_message>
feat(backend): complete Firebase cloud database migration for operations
</commit_message>
<xml_diff>
--- a/Progetto Scuole/rientri_ddt.xlsx
+++ b/Progetto Scuole/rientri_ddt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolution\dati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Il mio Drive\AppLogSolutions\Progetto Scuole\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42500EAC-F9D3-405C-B8F8-E161058D3536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA40B4BA-F4CB-4ABD-B7EC-179FDC4EF934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25540" yWindow="760" windowWidth="25660" windowHeight="12750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rientri" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="64">
   <si>
     <t>Codice consegna</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultColWidth="20.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.36328125" style="1" customWidth="1"/>
@@ -1096,15 +1096,18 @@
         <v>63</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>49</v>
       </c>
       <c r="B49" s="1">
         <v>46106</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>36</v>
       </c>
@@ -1112,15 +1115,18 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>50</v>
       </c>
       <c r="B51" s="1">
         <v>46106</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C51" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>40</v>
       </c>
@@ -1128,7 +1134,7 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>40</v>
       </c>
@@ -1136,7 +1142,7 @@
         <v>46099</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>51</v>
       </c>
@@ -1144,12 +1150,31 @@
         <v>46106</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>38</v>
       </c>
       <c r="B55" s="1">
         <v>46106</v>
+      </c>
+      <c r="C55" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" s="1">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>47</v>
+      </c>
+      <c r="B57" s="1">
+        <v>46107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>